<commit_message>
Updated PointPerformance to match Mission Profile
</commit_message>
<xml_diff>
--- a/Natsumi Excel Sheets/ASEN4138_ACDesign.xlsx
+++ b/Natsumi Excel Sheets/ASEN4138_ACDesign.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://o365coloradoedu-my.sharepoint.com/personal/aska7164_colorado_edu/Documents/Desktop/AES-AircraftDesignToolbox/MAIN/Input Excel Sheets/Design Configurations/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://o365coloradoedu-my.sharepoint.com/personal/aska7164_colorado_edu/Documents/Desktop/AC Design Code/MAIN/Input Excel Sheets/Design Configurations/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="41" documentId="13_ncr:1_{AF967D3A-6581-5D40-BFFA-E1DDAEB3102C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8F9FE5CF-C105-40D5-B6E0-DE4BBAFD673C}"/>
+  <xr:revisionPtr revIDLastSave="42" documentId="13_ncr:1_{AF967D3A-6581-5D40-BFFA-E1DDAEB3102C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{23C191F3-E7BA-4453-8231-62FA93387C51}"/>
   <bookViews>
-    <workbookView xWindow="2400" yWindow="1320" windowWidth="20640" windowHeight="12360" firstSheet="1" activeTab="3" xr2:uid="{904FC4B5-3CDE-421B-8E98-23A2C72E8C1E}"/>
+    <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="9960" firstSheet="1" activeTab="1" xr2:uid="{904FC4B5-3CDE-421B-8E98-23A2C72E8C1E}"/>
   </bookViews>
   <sheets>
     <sheet name="Variable Reference" sheetId="15" r:id="rId1"/>
@@ -3693,7 +3693,7 @@
         <v>1</v>
       </c>
       <c r="M4" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N4" s="4">
         <v>1209</v>

</xml_diff>